<commit_message>
Sync JR pipeline map, RA workpack, and ICMID coding updates.
Include cross-group map UX (detail panel, type filters, within-group records), JR_pair/RA workpack exports, ICMID Africa workbook, and literature sources for Dropbox sync.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/lookup/polygon_group_registry.xlsx
+++ b/data/lookup/polygon_group_registry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F133"/>
+  <dimension ref="A1:F153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3624,6 +3624,486 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ANGONI</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>greg</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Ngoni</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>TURKA</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Curama</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>IRAMBA</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Nyiramba</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>TIGRINYA</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Tigania</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>LUNGU</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Langulu</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>MAKUA</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Makoa</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>TATOGA</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Mangati</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>IRAQW</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Mbulu</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>TURU</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Nyaturu</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>MORU-MANGBETU AND SERE-MUNDU-SPEAKING PYGMY TRIBES</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>greg</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Mbuti</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>ESHIRA/BAPOUNOU</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>geopr</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Punu</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+      <c r="E144" t="inlineStr"/>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>EGEDE</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Imeggedezen</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>AHAGGAREN</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>all Tuareg</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>BIRA</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Bira villagers</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>DURU</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Dii</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>LUMBO</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Lumbu</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>MBEMBE</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Vingu</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>KUNYI</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Kugni</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>MAKONDE</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>murdock</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Mawia</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>SWAHILI</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>greg</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Vumba</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>synced from ethnic_entity_index</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sync ICMID unmatched sheet, Tuareg→GeoEPR, and map homeland fallback.
Drop Role/dedupe Unmatched entities; consolidate Tuareg to GeoEPR; use pipeline homeland columns when map resolver misses; keep only JR_pair sheet.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/lookup/polygon_group_registry.xlsx
+++ b/data/lookup/polygon_group_registry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F153"/>
+  <dimension ref="A1:F151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2955,7 +2955,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>TUAREGS</t>
+          <t>TUBU</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2965,7 +2965,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Tuaregs</t>
+          <t>Tubu</t>
         </is>
       </c>
       <c r="D106" t="inlineStr"/>
@@ -2979,17 +2979,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>TUBU</t>
+          <t>TUKULOR</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>greg</t>
+          <t>murdock</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Tubu</t>
+          <t>Tukulor</t>
         </is>
       </c>
       <c r="D107" t="inlineStr"/>
@@ -3003,7 +3003,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>TUKULOR</t>
+          <t>TUMBUKA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Tukulor</t>
+          <t>Tumbuka</t>
         </is>
       </c>
       <c r="D108" t="inlineStr"/>
@@ -3027,7 +3027,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>TUMBUKA</t>
+          <t>TURKANA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Tumbuka</t>
+          <t>Turkana</t>
         </is>
       </c>
       <c r="D109" t="inlineStr"/>
@@ -3051,7 +3051,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>TURKANA</t>
+          <t>TUSYAN</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Turkana</t>
+          <t>Tusyan</t>
         </is>
       </c>
       <c r="D110" t="inlineStr"/>
@@ -3075,7 +3075,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>TUSYAN</t>
+          <t>VENDA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Tusyan</t>
+          <t>Venda</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
@@ -3099,7 +3099,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>VENDA</t>
+          <t>WARA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Venda</t>
+          <t>Wara</t>
         </is>
       </c>
       <c r="D112" t="inlineStr"/>
@@ -3123,7 +3123,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>WARA</t>
+          <t>WOLOF</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Wara</t>
+          <t>Wolof</t>
         </is>
       </c>
       <c r="D113" t="inlineStr"/>
@@ -3147,7 +3147,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>WOLOF</t>
+          <t>YAO</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3157,7 +3157,7 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Wolof</t>
+          <t>Yao</t>
         </is>
       </c>
       <c r="D114" t="inlineStr"/>
@@ -3171,7 +3171,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>YAO</t>
+          <t>YORUBA</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3181,7 +3181,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Yao</t>
+          <t>Yoruba</t>
         </is>
       </c>
       <c r="D115" t="inlineStr"/>
@@ -3195,7 +3195,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>YORUBA</t>
+          <t>ZARAMO</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Yoruba</t>
+          <t>Zaramo</t>
         </is>
       </c>
       <c r="D116" t="inlineStr"/>
@@ -3219,7 +3219,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ZARAMO</t>
+          <t>ZERMA</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Zaramo</t>
+          <t>Zerma</t>
         </is>
       </c>
       <c r="D117" t="inlineStr"/>
@@ -3243,7 +3243,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ZERMA</t>
+          <t>ZULU</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Zerma</t>
+          <t>Zulu</t>
         </is>
       </c>
       <c r="D118" t="inlineStr"/>
@@ -3267,31 +3267,31 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ZULU</t>
+          <t>PEUL</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>murdock</t>
+          <t>geopr</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Zulu</t>
+          <t>Peul</t>
         </is>
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
-          <t>bootstrapped from entity index polygon_ids</t>
+          <t>synced from ethnic_entity_index</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>PEUL</t>
+          <t>KANOURI</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3301,7 +3301,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Peul</t>
+          <t>Kanouri</t>
         </is>
       </c>
       <c r="D120" t="inlineStr"/>
@@ -3315,7 +3315,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>KANOURI</t>
+          <t>MANDINKA</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3325,7 +3325,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Kanouri</t>
+          <t>Mandinka</t>
         </is>
       </c>
       <c r="D121" t="inlineStr"/>
@@ -3339,17 +3339,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MANDINKA</t>
+          <t>ZIGULA</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>geopr</t>
+          <t>murdock</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Mandinka</t>
+          <t>Zigua</t>
         </is>
       </c>
       <c r="D122" t="inlineStr"/>
@@ -3363,7 +3363,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ZIGULA</t>
+          <t>BIRIFON</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3373,7 +3373,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Zigua</t>
+          <t>Birifor</t>
         </is>
       </c>
       <c r="D123" t="inlineStr"/>
@@ -3387,17 +3387,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>BIRIFON</t>
+          <t>MORO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>murdock</t>
+          <t>geopr</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Birifor</t>
+          <t>Moro</t>
         </is>
       </c>
       <c r="D124" t="inlineStr"/>
@@ -3411,7 +3411,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>MORO</t>
+          <t>NUBA</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Moro</t>
+          <t>Nuba</t>
         </is>
       </c>
       <c r="D125" t="inlineStr"/>
@@ -3435,7 +3435,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>NUBA</t>
+          <t>SOMALI</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Nuba</t>
+          <t>Somali</t>
         </is>
       </c>
       <c r="D126" t="inlineStr"/>
@@ -3459,7 +3459,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>SOMALI</t>
+          <t>TUAREG</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3469,21 +3469,25 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Somali</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr"/>
+          <t>Tuareg</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>AHAGGAREN, Ahaggaren, Tuaregs, all Tuareg, noble Tuareg</t>
+        </is>
+      </c>
       <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
-          <t>synced from ethnic_entity_index</t>
+          <t>GeoEPR Tuareg homeland; consolidated from GREG Tuaregs / Murdock AHAGGAREN</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>TUAREG</t>
+          <t>INDIGENOUS LOWLAND PEOPLES (SHUAR, ACHUAR ETC.)</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3493,7 +3497,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Tuareg</t>
+          <t>all the clans with plant names</t>
         </is>
       </c>
       <c r="D128" t="inlineStr"/>
@@ -3507,7 +3511,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>INDIGENOUS LOWLAND PEOPLES (SHUAR, ACHUAR ETC.)</t>
+          <t>OTHER INDIGENOUS GROUPS</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3517,7 +3521,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>all the clans with plant names</t>
+          <t>her</t>
         </is>
       </c>
       <c r="D129" t="inlineStr"/>
@@ -3531,7 +3535,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>OTHER INDIGENOUS GROUPS</t>
+          <t>PASHTUNS</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3541,7 +3545,7 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>her</t>
+          <t>tun</t>
         </is>
       </c>
       <c r="D130" t="inlineStr"/>
@@ -3555,17 +3559,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PASHTUNS</t>
+          <t>GURMA</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>geopr</t>
+          <t>murdock</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>tun</t>
+          <t>Gourmantché</t>
         </is>
       </c>
       <c r="D131" t="inlineStr"/>
@@ -3579,7 +3583,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>GURMA</t>
+          <t>LILSE</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3589,7 +3593,7 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Gourmantché</t>
+          <t>Kurumba</t>
         </is>
       </c>
       <c r="D132" t="inlineStr"/>
@@ -3603,17 +3607,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>LILSE</t>
+          <t>ANGONI</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>murdock</t>
+          <t>greg</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Kurumba</t>
+          <t>Ngoni</t>
         </is>
       </c>
       <c r="D133" t="inlineStr"/>
@@ -3627,17 +3631,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ANGONI</t>
+          <t>TURKA</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>greg</t>
+          <t>murdock</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Ngoni</t>
+          <t>Curama</t>
         </is>
       </c>
       <c r="D134" t="inlineStr"/>
@@ -3651,7 +3655,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>TURKA</t>
+          <t>IRAMBA</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -3661,7 +3665,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Curama</t>
+          <t>Nyiramba</t>
         </is>
       </c>
       <c r="D135" t="inlineStr"/>
@@ -3675,7 +3679,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IRAMBA</t>
+          <t>TIGRINYA</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3685,7 +3689,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Nyiramba</t>
+          <t>Tigania</t>
         </is>
       </c>
       <c r="D136" t="inlineStr"/>
@@ -3699,7 +3703,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>TIGRINYA</t>
+          <t>LUNGU</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3709,7 +3713,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Tigania</t>
+          <t>Langulu</t>
         </is>
       </c>
       <c r="D137" t="inlineStr"/>
@@ -3723,7 +3727,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LUNGU</t>
+          <t>MAKUA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3733,7 +3737,7 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Langulu</t>
+          <t>Makoa</t>
         </is>
       </c>
       <c r="D138" t="inlineStr"/>
@@ -3747,7 +3751,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>MAKUA</t>
+          <t>TATOGA</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -3757,7 +3761,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Makoa</t>
+          <t>Mangati</t>
         </is>
       </c>
       <c r="D139" t="inlineStr"/>
@@ -3771,7 +3775,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>TATOGA</t>
+          <t>IRAQW</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3781,7 +3785,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Mangati</t>
+          <t>Mbulu</t>
         </is>
       </c>
       <c r="D140" t="inlineStr"/>
@@ -3795,7 +3799,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>IRAQW</t>
+          <t>TURU</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3805,7 +3809,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Mbulu</t>
+          <t>Nyaturu</t>
         </is>
       </c>
       <c r="D141" t="inlineStr"/>
@@ -3819,17 +3823,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>TURU</t>
+          <t>MORU-MANGBETU AND SERE-MUNDU-SPEAKING PYGMY TRIBES</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>murdock</t>
+          <t>greg</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Nyaturu</t>
+          <t>Mbuti</t>
         </is>
       </c>
       <c r="D142" t="inlineStr"/>
@@ -3843,17 +3847,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>MORU-MANGBETU AND SERE-MUNDU-SPEAKING PYGMY TRIBES</t>
+          <t>ESHIRA/BAPOUNOU</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>greg</t>
+          <t>geopr</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Mbuti</t>
+          <t>Punu</t>
         </is>
       </c>
       <c r="D143" t="inlineStr"/>
@@ -3867,17 +3871,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ESHIRA/BAPOUNOU</t>
+          <t>EGEDE</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>geopr</t>
+          <t>murdock</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Punu</t>
+          <t>Imeggedezen</t>
         </is>
       </c>
       <c r="D144" t="inlineStr"/>
@@ -3891,7 +3895,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>EGEDE</t>
+          <t>BIRA</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3901,7 +3905,7 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Imeggedezen</t>
+          <t>Bira villagers</t>
         </is>
       </c>
       <c r="D145" t="inlineStr"/>
@@ -3915,7 +3919,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>AHAGGAREN</t>
+          <t>DURU</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3925,7 +3929,7 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>all Tuareg</t>
+          <t>Dii</t>
         </is>
       </c>
       <c r="D146" t="inlineStr"/>
@@ -3939,7 +3943,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>BIRA</t>
+          <t>LUMBO</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -3949,7 +3953,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Bira villagers</t>
+          <t>Lumbu</t>
         </is>
       </c>
       <c r="D147" t="inlineStr"/>
@@ -3963,7 +3967,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>DURU</t>
+          <t>MBEMBE</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -3973,7 +3977,7 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Dii</t>
+          <t>Vingu</t>
         </is>
       </c>
       <c r="D148" t="inlineStr"/>
@@ -3987,7 +3991,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>LUMBO</t>
+          <t>KUNYI</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -3997,7 +4001,7 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Lumbu</t>
+          <t>Kugni</t>
         </is>
       </c>
       <c r="D149" t="inlineStr"/>
@@ -4011,7 +4015,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MBEMBE</t>
+          <t>MAKONDE</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4021,7 +4025,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Vingu</t>
+          <t>Mawia</t>
         </is>
       </c>
       <c r="D150" t="inlineStr"/>
@@ -4035,70 +4039,22 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>KUNYI</t>
+          <t>SWAHILI</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>murdock</t>
+          <t>greg</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Kugni</t>
+          <t>Vumba</t>
         </is>
       </c>
       <c r="D151" t="inlineStr"/>
       <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
-        <is>
-          <t>synced from ethnic_entity_index</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>MAKONDE</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>murdock</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Mawia</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr"/>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr">
-        <is>
-          <t>synced from ethnic_entity_index</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>SWAHILI</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>greg</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>Vumba</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr"/>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr">
         <is>
           <t>synced from ethnic_entity_index</t>
         </is>

</xml_diff>